<commit_message>
add annual growth per sector
</commit_message>
<xml_diff>
--- a/DeskripsiSektor.xlsx
+++ b/DeskripsiSektor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy-GGP-PNG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B42F943-8649-4E5A-9C64-538CFB194581}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0157684C-C261-47C7-BE05-5988A7654BD8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
   </bookViews>
@@ -41,41 +41,6 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Bodro, Dewi Kiswani</author>
-  </authors>
-  <commentList>
-    <comment ref="G18" authorId="0" shapeId="0" xr:uid="{655ECD27-9EAB-49DE-92FE-65BADE35BEF0}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Bodro, Dewi Kiswani:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Asumsi sementara untuk running data
-</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="91">
   <si>
@@ -356,26 +321,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -433,7 +385,8 @@
       <sheetName val="Oro_2019 (cek)"/>
       <sheetName val="Oro_2023 (cek)"/>
       <sheetName val="List Data Input"/>
-      <sheetName val="io"/>
+      <sheetName val="io 2019"/>
+      <sheetName val="io 2023"/>
       <sheetName val="DeskripsiSektor"/>
       <sheetName val="LDC"/>
       <sheetName val="BAU_Lahan"/>
@@ -453,7 +406,8 @@
       <sheetData sheetId="8"/>
       <sheetData sheetId="9"/>
       <sheetData sheetId="10"/>
-      <sheetData sheetId="11">
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12">
         <row r="2">
           <cell r="D2">
             <v>100.69717125</v>
@@ -660,8 +614,8 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="12"/>
       <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -983,7 +937,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51CCBCFD-2E22-41F3-84DE-C40DB9077DD2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51CCBCFD-2E22-41F3-84DE-C40DB9077DD2}">
   <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1475,7 +1429,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="H18" s="2">
         <f>[1]TK!D18</f>
@@ -1502,7 +1456,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>-0.15810000000000002</v>
       </c>
       <c r="H19" s="2">
         <f>[1]TK!D19</f>
@@ -1529,7 +1483,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.35930000000000001</v>
       </c>
       <c r="H20" s="2">
         <f>[1]TK!D20</f>
@@ -1556,7 +1510,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.1993</v>
       </c>
       <c r="H21" s="2">
         <f>[1]TK!D21</f>
@@ -1583,7 +1537,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>2.52E-2</v>
       </c>
       <c r="H22" s="2">
         <f>[1]TK!D22</f>
@@ -1610,7 +1564,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.65749999999999997</v>
       </c>
       <c r="H23" s="2">
         <f>[1]TK!D23</f>
@@ -1637,7 +1591,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="H24" s="2">
         <f>[1]TK!D24</f>
@@ -1664,7 +1618,7 @@
         <v>1</v>
       </c>
       <c r="G25" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.5474</v>
       </c>
       <c r="H25" s="2">
         <f>[1]TK!D25</f>
@@ -1691,7 +1645,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.44659999999999994</v>
       </c>
       <c r="H26" s="2">
         <f>[1]TK!D26</f>
@@ -1718,7 +1672,7 @@
         <v>1</v>
       </c>
       <c r="G27" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>-0.57779999999999998</v>
       </c>
       <c r="H27" s="2">
         <f>[1]TK!D27</f>
@@ -1745,7 +1699,7 @@
         <v>1</v>
       </c>
       <c r="G28" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>8.6699999999999999E-2</v>
       </c>
       <c r="H28" s="2">
         <f>[1]TK!D28</f>
@@ -1772,7 +1726,7 @@
         <v>1</v>
       </c>
       <c r="G29" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>5.16E-2</v>
       </c>
       <c r="H29" s="2">
         <f>[1]TK!D29</f>
@@ -1799,7 +1753,7 @@
         <v>1</v>
       </c>
       <c r="G30" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.15179999999999999</v>
       </c>
       <c r="H30" s="2">
         <f>[1]TK!D30</f>
@@ -1826,7 +1780,7 @@
         <v>1</v>
       </c>
       <c r="G31" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>-0.40399999999999997</v>
       </c>
       <c r="H31" s="2">
         <f>[1]TK!D31</f>
@@ -1853,7 +1807,7 @@
         <v>1</v>
       </c>
       <c r="G32" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>-0.15990000000000001</v>
       </c>
       <c r="H32" s="2">
         <f>[1]TK!D32</f>
@@ -1880,7 +1834,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>6.0299999999999999E-2</v>
       </c>
       <c r="H33" s="2">
         <f>[1]TK!D33</f>
@@ -1907,7 +1861,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.18530000000000002</v>
       </c>
       <c r="H34" s="2">
         <f>[1]TK!D34</f>
@@ -1934,7 +1888,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>4.0099999999999997E-2</v>
       </c>
       <c r="H35" s="2">
         <f>[1]TK!D35</f>
@@ -1961,7 +1915,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.17929999999999999</v>
       </c>
       <c r="H36" s="2">
         <f>[1]TK!D36</f>
@@ -1988,7 +1942,7 @@
         <v>1</v>
       </c>
       <c r="G37" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>9.3699999999999992E-2</v>
       </c>
       <c r="H37" s="2">
         <f>[1]TK!D37</f>
@@ -2015,7 +1969,7 @@
         <v>1</v>
       </c>
       <c r="G38" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.1032</v>
       </c>
       <c r="H38" s="2">
         <f>[1]TK!D38</f>
@@ -2042,7 +1996,7 @@
         <v>1</v>
       </c>
       <c r="G39" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>5.3899999999999997E-2</v>
       </c>
       <c r="H39" s="2">
         <f>[1]TK!D39</f>
@@ -2069,7 +2023,7 @@
         <v>1</v>
       </c>
       <c r="G40" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0.08</v>
       </c>
       <c r="H40" s="2">
         <f>[1]TK!D40</f>
@@ -2096,7 +2050,7 @@
         <v>1</v>
       </c>
       <c r="G41" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>2.3900000000000001E-2</v>
       </c>
       <c r="H41" s="2">
         <f>[1]TK!D41</f>
@@ -2123,7 +2077,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="H42" s="2">
         <f>[1]TK!D42</f>
@@ -2132,6 +2086,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ubah pembagi jadi total output dan pdrb dibatasi max dan min
</commit_message>
<xml_diff>
--- a/DeskripsiSektor.xlsx
+++ b/DeskripsiSektor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy-GGP-PNG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0157684C-C261-47C7-BE05-5988A7654BD8}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{012F7B52-9B6E-4DAD-A204-1E94FA6EBA3E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
+    <workbookView minimized="1" xWindow="5436" yWindow="4860" windowWidth="17280" windowHeight="9960" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
   </bookViews>
   <sheets>
     <sheet name="DeskripsiSektor" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
use X_prov (TotalInput) and RateUnconstrained  mean 1%
</commit_message>
<xml_diff>
--- a/DeskripsiSektor.xlsx
+++ b/DeskripsiSektor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy-GGP-PNG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{012F7B52-9B6E-4DAD-A204-1E94FA6EBA3E}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E0EB8F7-61B4-484D-A14F-E5CBEC3B3C09}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5436" yWindow="4860" windowWidth="17280" windowHeight="9960" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
   </bookViews>
   <sheets>
     <sheet name="DeskripsiSektor" sheetId="1" r:id="rId1"/>
@@ -321,7 +321,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -347,15 +358,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -392,7 +405,8 @@
       <sheetName val="BAU_Lahan"/>
       <sheetName val="TK"/>
       <sheetName val="Assumption_TK"/>
-      <sheetName val="Sheet6"/>
+      <sheetName val="GrowthUncons_Calc"/>
+      <sheetName val="GrowthUncons_Calc_PNG"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -616,6 +630,7 @@
       </sheetData>
       <sheetData sheetId="13"/>
       <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -999,7 +1014,7 @@
       <c r="G2">
         <v>0</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <f>[1]TK!D2</f>
         <v>100.69717125</v>
       </c>
@@ -1026,7 +1041,7 @@
       <c r="G3">
         <v>0</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <f>[1]TK!D3</f>
         <v>201.39434249999999</v>
       </c>
@@ -1053,7 +1068,7 @@
       <c r="G4">
         <v>0</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <f>[1]TK!D4</f>
         <v>201.39434249999999</v>
       </c>
@@ -1080,7 +1095,7 @@
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <f>[1]TK!D5</f>
         <v>201.39434249999999</v>
       </c>
@@ -1107,7 +1122,7 @@
       <c r="G6">
         <v>0</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <f>[1]TK!D6</f>
         <v>12003.102813</v>
       </c>
@@ -1134,7 +1149,7 @@
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <f>[1]TK!D7</f>
         <v>30007.757032499998</v>
       </c>
@@ -1161,7 +1176,7 @@
       <c r="G8">
         <v>0</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <f>[1]TK!D8</f>
         <v>7995.3553972499994</v>
       </c>
@@ -1188,7 +1203,7 @@
       <c r="G9">
         <v>0</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <f>[1]TK!D9</f>
         <v>503.48585624999998</v>
       </c>
@@ -1215,7 +1230,7 @@
       <c r="G10">
         <v>0</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <f>[1]TK!D10</f>
         <v>6998.453401875001</v>
       </c>
@@ -1242,7 +1257,7 @@
       <c r="G11">
         <v>0</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <f>[1]TK!D11</f>
         <v>1500.3878516249999</v>
       </c>
@@ -1269,7 +1284,7 @@
       <c r="G12">
         <v>0</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <f>[1]TK!D12</f>
         <v>5034.8585625000005</v>
       </c>
@@ -1296,7 +1311,7 @@
       <c r="G13">
         <v>0</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <f>[1]TK!D13</f>
         <v>2003.873707875</v>
       </c>
@@ -1323,7 +1338,7 @@
       <c r="G14">
         <v>0</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <f>[1]TK!D14</f>
         <v>1500.3878516249999</v>
       </c>
@@ -1350,7 +1365,7 @@
       <c r="G15">
         <v>0</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <f>[1]TK!D15</f>
         <v>503.48585624999998</v>
       </c>
@@ -1377,7 +1392,7 @@
       <c r="G16">
         <v>0</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <f>[1]TK!D16</f>
         <v>805.57736999999997</v>
       </c>
@@ -1404,7 +1419,7 @@
       <c r="G17">
         <v>0</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <f>[1]TK!D17</f>
         <v>3524.4009937500005</v>
       </c>
@@ -1428,10 +1443,10 @@
       <c r="F18">
         <v>1</v>
       </c>
-      <c r="G18" s="1">
+      <c r="G18" s="2">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <f>[1]TK!D18</f>
         <v>302.09151374999999</v>
       </c>
@@ -1455,10 +1470,10 @@
       <c r="F19">
         <v>1</v>
       </c>
-      <c r="G19" s="1">
-        <v>-0.15810000000000002</v>
-      </c>
-      <c r="H19" s="2">
+      <c r="G19" s="2">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1">
         <f>[1]TK!D19</f>
         <v>1500.3878516249999</v>
       </c>
@@ -1482,10 +1497,10 @@
       <c r="F20">
         <v>1</v>
       </c>
-      <c r="G20" s="1">
-        <v>0.35930000000000001</v>
-      </c>
-      <c r="H20" s="2">
+      <c r="G20" s="2">
+        <v>0.41808508590274895</v>
+      </c>
+      <c r="H20" s="1">
         <f>[1]TK!D20</f>
         <v>201.39434249999999</v>
       </c>
@@ -1509,10 +1524,10 @@
       <c r="F21">
         <v>1</v>
       </c>
-      <c r="G21" s="1">
-        <v>0.1993</v>
-      </c>
-      <c r="H21" s="2">
+      <c r="G21" s="2">
+        <v>0</v>
+      </c>
+      <c r="H21" s="1">
         <f>[1]TK!D21</f>
         <v>100.69717125</v>
       </c>
@@ -1536,10 +1551,10 @@
       <c r="F22">
         <v>1</v>
       </c>
-      <c r="G22" s="1">
-        <v>2.52E-2</v>
-      </c>
-      <c r="H22" s="2">
+      <c r="G22" s="2">
+        <v>1.1474827820314282E-2</v>
+      </c>
+      <c r="H22" s="1">
         <f>[1]TK!D22</f>
         <v>402.78868499999999</v>
       </c>
@@ -1563,10 +1578,10 @@
       <c r="F23">
         <v>1</v>
       </c>
-      <c r="G23" s="1">
-        <v>0.65749999999999997</v>
-      </c>
-      <c r="H23" s="2">
+      <c r="G23" s="2">
+        <v>0.10204164174912744</v>
+      </c>
+      <c r="H23" s="1">
         <f>[1]TK!D23</f>
         <v>50.348585624999998</v>
       </c>
@@ -1590,10 +1605,10 @@
       <c r="F24">
         <v>1</v>
       </c>
-      <c r="G24" s="1">
-        <v>0</v>
-      </c>
-      <c r="H24" s="2">
+      <c r="G24" s="2">
+        <v>0.2225185103524232</v>
+      </c>
+      <c r="H24" s="1">
         <f>[1]TK!D24</f>
         <v>100.69717125</v>
       </c>
@@ -1617,10 +1632,10 @@
       <c r="F25">
         <v>1</v>
       </c>
-      <c r="G25" s="1">
-        <v>0.5474</v>
-      </c>
-      <c r="H25" s="2">
+      <c r="G25" s="2">
+        <v>0.71908987139005265</v>
+      </c>
+      <c r="H25" s="1">
         <f>[1]TK!D25</f>
         <v>50.348585624999998</v>
       </c>
@@ -1644,10 +1659,10 @@
       <c r="F26">
         <v>1</v>
       </c>
-      <c r="G26" s="1">
-        <v>0.44659999999999994</v>
-      </c>
-      <c r="H26" s="2">
+      <c r="G26" s="2">
+        <v>0</v>
+      </c>
+      <c r="H26" s="1">
         <f>[1]TK!D26</f>
         <v>50.348585624999998</v>
       </c>
@@ -1671,10 +1686,10 @@
       <c r="F27">
         <v>1</v>
       </c>
-      <c r="G27" s="1">
-        <v>-0.57779999999999998</v>
-      </c>
-      <c r="H27" s="2">
+      <c r="G27" s="2">
+        <v>0</v>
+      </c>
+      <c r="H27" s="1">
         <f>[1]TK!D27</f>
         <v>201.39434249999999</v>
       </c>
@@ -1698,10 +1713,10 @@
       <c r="F28">
         <v>1</v>
       </c>
-      <c r="G28" s="1">
-        <v>8.6699999999999999E-2</v>
-      </c>
-      <c r="H28" s="2">
+      <c r="G28" s="2">
+        <v>6.9332659657442175E-2</v>
+      </c>
+      <c r="H28" s="1">
         <f>[1]TK!D28</f>
         <v>302.09151374999999</v>
       </c>
@@ -1725,10 +1740,10 @@
       <c r="F29">
         <v>1</v>
       </c>
-      <c r="G29" s="1">
-        <v>5.16E-2</v>
-      </c>
-      <c r="H29" s="2">
+      <c r="G29" s="2">
+        <v>0.20272920751195733</v>
+      </c>
+      <c r="H29" s="1">
         <f>[1]TK!D29</f>
         <v>201.39434249999999</v>
       </c>
@@ -1752,10 +1767,10 @@
       <c r="F30">
         <v>1</v>
       </c>
-      <c r="G30" s="1">
-        <v>0.15179999999999999</v>
-      </c>
-      <c r="H30" s="2">
+      <c r="G30" s="2">
+        <v>0.15619685398174643</v>
+      </c>
+      <c r="H30" s="1">
         <f>[1]TK!D30</f>
         <v>2003.873707875</v>
       </c>
@@ -1779,10 +1794,10 @@
       <c r="F31">
         <v>1</v>
       </c>
-      <c r="G31" s="1">
-        <v>-0.40399999999999997</v>
-      </c>
-      <c r="H31" s="2">
+      <c r="G31" s="2">
+        <v>7.9160750938956248E-2</v>
+      </c>
+      <c r="H31" s="1">
         <f>[1]TK!D31</f>
         <v>5004.6494111250004</v>
       </c>
@@ -1806,10 +1821,10 @@
       <c r="F32">
         <v>1</v>
       </c>
-      <c r="G32" s="1">
-        <v>-0.15990000000000001</v>
-      </c>
-      <c r="H32" s="2">
+      <c r="G32" s="2">
+        <v>3.3716767936662118E-2</v>
+      </c>
+      <c r="H32" s="1">
         <f>[1]TK!D32</f>
         <v>2497.289847</v>
       </c>
@@ -1833,10 +1848,10 @@
       <c r="F33">
         <v>1</v>
       </c>
-      <c r="G33" s="1">
-        <v>6.0299999999999999E-2</v>
-      </c>
-      <c r="H33" s="2">
+      <c r="G33" s="2">
+        <v>5.6907034608510099E-2</v>
+      </c>
+      <c r="H33" s="1">
         <f>[1]TK!D33</f>
         <v>503.48585624999998</v>
       </c>
@@ -1860,10 +1875,10 @@
       <c r="F34">
         <v>1</v>
       </c>
-      <c r="G34" s="1">
-        <v>0.18530000000000002</v>
-      </c>
-      <c r="H34" s="2">
+      <c r="G34" s="2">
+        <v>0.12868594096542441</v>
+      </c>
+      <c r="H34" s="1">
         <f>[1]TK!D34</f>
         <v>302.09151374999999</v>
       </c>
@@ -1887,10 +1902,10 @@
       <c r="F35">
         <v>1</v>
       </c>
-      <c r="G35" s="1">
-        <v>4.0099999999999997E-2</v>
-      </c>
-      <c r="H35" s="2">
+      <c r="G35" s="2">
+        <v>0</v>
+      </c>
+      <c r="H35" s="1">
         <f>[1]TK!D35</f>
         <v>402.78868499999999</v>
       </c>
@@ -1914,10 +1929,10 @@
       <c r="F36">
         <v>1</v>
       </c>
-      <c r="G36" s="1">
-        <v>0.17929999999999999</v>
-      </c>
-      <c r="H36" s="2">
+      <c r="G36" s="2">
+        <v>0.18185073335734003</v>
+      </c>
+      <c r="H36" s="1">
         <f>[1]TK!D36</f>
         <v>151.045756875</v>
       </c>
@@ -1941,10 +1956,10 @@
       <c r="F37">
         <v>1</v>
       </c>
-      <c r="G37" s="1">
-        <v>9.3699999999999992E-2</v>
-      </c>
-      <c r="H37" s="2">
+      <c r="G37" s="2">
+        <v>4.424127182093418E-2</v>
+      </c>
+      <c r="H37" s="1">
         <f>[1]TK!D37</f>
         <v>503.48585624999998</v>
       </c>
@@ -1968,10 +1983,10 @@
       <c r="F38">
         <v>1</v>
       </c>
-      <c r="G38" s="1">
-        <v>0.1032</v>
-      </c>
-      <c r="H38" s="2">
+      <c r="G38" s="2">
+        <v>9.8798245163341791E-2</v>
+      </c>
+      <c r="H38" s="1">
         <f>[1]TK!D38</f>
         <v>3000.7757032499999</v>
       </c>
@@ -1995,10 +2010,10 @@
       <c r="F39">
         <v>1</v>
       </c>
-      <c r="G39" s="1">
-        <v>5.3899999999999997E-2</v>
-      </c>
-      <c r="H39" s="2">
+      <c r="G39" s="2">
+        <v>6.5439809491808498E-2</v>
+      </c>
+      <c r="H39" s="1">
         <f>[1]TK!D39</f>
         <v>2497.289847</v>
       </c>
@@ -2022,10 +2037,10 @@
       <c r="F40">
         <v>1</v>
       </c>
-      <c r="G40" s="1">
-        <v>0.08</v>
-      </c>
-      <c r="H40" s="2">
+      <c r="G40" s="2">
+        <v>7.826757953253205E-2</v>
+      </c>
+      <c r="H40" s="1">
         <f>[1]TK!D40</f>
         <v>1198.2963378750001</v>
       </c>
@@ -2049,10 +2064,10 @@
       <c r="F41">
         <v>1</v>
       </c>
-      <c r="G41" s="1">
+      <c r="G41" s="2">
         <v>2.3900000000000001E-2</v>
       </c>
-      <c r="H41" s="2">
+      <c r="H41" s="1">
         <f>[1]TK!D41</f>
         <v>2497.289847</v>
       </c>
@@ -2076,10 +2091,10 @@
       <c r="F42">
         <v>1</v>
       </c>
-      <c r="G42" s="1">
-        <v>0</v>
-      </c>
-      <c r="H42" s="2">
+      <c r="G42" s="2">
+        <v>0</v>
+      </c>
+      <c r="H42" s="1">
         <f>[1]TK!D42</f>
         <v>3584.8192964999998</v>
       </c>

</xml_diff>

<commit_message>
agregate sector (peleburan sektor yang tidak sig)
</commit_message>
<xml_diff>
--- a/DeskripsiSektor.xlsx
+++ b/DeskripsiSektor.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy-GGP-PNG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E0EB8F7-61B4-484D-A14F-E5CBEC3B3C09}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0D032CE-CAB2-4934-82A0-FD6136D6581B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
   </bookViews>
   <sheets>
     <sheet name="DeskripsiSektor" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="90">
   <si>
     <t>KodeSektor</t>
   </si>
@@ -68,36 +65,18 @@
     <t>TenagaKerja</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>cmaiz</t>
   </si>
   <si>
     <t>crice</t>
   </si>
   <si>
-    <t>cocer</t>
-  </si>
-  <si>
-    <t>cpuls</t>
-  </si>
-  <si>
     <t>coils</t>
   </si>
   <si>
-    <t>croot</t>
-  </si>
-  <si>
-    <t>cvege</t>
-  </si>
-  <si>
     <t>csugr</t>
   </si>
   <si>
-    <t>cfrui</t>
-  </si>
-  <si>
     <t>ccoff</t>
   </si>
   <si>
@@ -128,9 +107,6 @@
     <t>cbeve</t>
   </si>
   <si>
-    <t>ctext</t>
-  </si>
-  <si>
     <t>cwood</t>
   </si>
   <si>
@@ -158,12 +134,6 @@
     <t>ccons</t>
   </si>
   <si>
-    <t>ctrad</t>
-  </si>
-  <si>
-    <t>ctran</t>
-  </si>
-  <si>
     <t>chotl</t>
   </si>
   <si>
@@ -191,33 +161,15 @@
     <t>cosrv</t>
   </si>
   <si>
-    <t>Maize</t>
-  </si>
-  <si>
     <t>Rice</t>
   </si>
   <si>
-    <t>Other cereals</t>
-  </si>
-  <si>
-    <t>Pulses</t>
-  </si>
-  <si>
     <t>Oilseeds</t>
   </si>
   <si>
-    <t>Roots</t>
-  </si>
-  <si>
-    <t>Vegetables</t>
-  </si>
-  <si>
     <t>Sugarcane</t>
   </si>
   <si>
-    <t>Fruits and nuts</t>
-  </si>
-  <si>
     <t>Coffee, tea and cocoa</t>
   </si>
   <si>
@@ -248,9 +200,6 @@
     <t>Beverage and tobacco</t>
   </si>
   <si>
-    <t>Textiles, clothing and footwear</t>
-  </si>
-  <si>
     <t>Wood and paper products</t>
   </si>
   <si>
@@ -266,9 +215,6 @@
     <t>Machinery, equipment and vehicles</t>
   </si>
   <si>
-    <t>Other manufacturing</t>
-  </si>
-  <si>
     <t>Electricity, gas and steam</t>
   </si>
   <si>
@@ -278,12 +224,6 @@
     <t>Construction</t>
   </si>
   <si>
-    <t>Wholesale and retail trade</t>
-  </si>
-  <si>
-    <t>Transportation and storage</t>
-  </si>
-  <si>
     <t>Accommodation and food services</t>
   </si>
   <si>
@@ -315,6 +255,60 @@
   </si>
   <si>
     <t>coesub</t>
+  </si>
+  <si>
+    <t>Maiz, Pulses, Other Cereals</t>
+  </si>
+  <si>
+    <t>Agriculture, Forestry and Fishery</t>
+  </si>
+  <si>
+    <t>Horticulture (Vegetables, Roots, fruits and nuts)</t>
+  </si>
+  <si>
+    <t>Mining and Quarrying</t>
+  </si>
+  <si>
+    <t>Manufacturing Industry</t>
+  </si>
+  <si>
+    <t>Other manufacturing include textile, clothing, and footware</t>
+  </si>
+  <si>
+    <t>Electricity and Gas Supply</t>
+  </si>
+  <si>
+    <t>Water Supply, Waste Management and Remediation</t>
+  </si>
+  <si>
+    <t>Accommodation and Food Service Activities</t>
+  </si>
+  <si>
+    <t>Information and Communication</t>
+  </si>
+  <si>
+    <t>Financial and Insurance Activities</t>
+  </si>
+  <si>
+    <t>Real Estate Activities</t>
+  </si>
+  <si>
+    <t>Business Services</t>
+  </si>
+  <si>
+    <t>Public Administration, Defence and Social Security</t>
+  </si>
+  <si>
+    <t>Education Services</t>
+  </si>
+  <si>
+    <t>Human Health and Social Work Activities</t>
+  </si>
+  <si>
+    <t>Other Services</t>
+  </si>
+  <si>
+    <t>Other Services / Unclassified</t>
   </si>
 </sst>
 </file>
@@ -323,7 +317,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -365,7 +359,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -382,258 +376,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Oro_2019_IO"/>
-      <sheetName val="Oro_2023_IO"/>
-      <sheetName val="PNG_2019_IO"/>
-      <sheetName val="PNG_2023_IO"/>
-      <sheetName val="Oro_2019 (cek)"/>
-      <sheetName val="Oro_2023 (cek)"/>
-      <sheetName val="List Data Input"/>
-      <sheetName val="io 2019"/>
-      <sheetName val="io 2023"/>
-      <sheetName val="DeskripsiSektor"/>
-      <sheetName val="LDC"/>
-      <sheetName val="BAU_Lahan"/>
-      <sheetName val="TK"/>
-      <sheetName val="Assumption_TK"/>
-      <sheetName val="GrowthUncons_Calc"/>
-      <sheetName val="GrowthUncons_Calc_PNG"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12">
-        <row r="2">
-          <cell r="D2">
-            <v>100.69717125</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="D3">
-            <v>201.39434249999999</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="D4">
-            <v>201.39434249999999</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="D5">
-            <v>201.39434249999999</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="D6">
-            <v>12003.102813</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="D7">
-            <v>30007.757032499998</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="D8">
-            <v>7995.3553972499994</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="D9">
-            <v>503.48585624999998</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="D10">
-            <v>6998.453401875001</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="D11">
-            <v>1500.3878516249999</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="D12">
-            <v>5034.8585625000005</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="D13">
-            <v>2003.873707875</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="D14">
-            <v>1500.3878516249999</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="D15">
-            <v>503.48585624999998</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="D16">
-            <v>805.57736999999997</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="D17">
-            <v>3524.4009937500005</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="D18">
-            <v>302.09151374999999</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="D19">
-            <v>1500.3878516249999</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="D20">
-            <v>201.39434249999999</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="D21">
-            <v>100.69717125</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="D22">
-            <v>402.78868499999999</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="D23">
-            <v>50.348585624999998</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="D24">
-            <v>100.69717125</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="D25">
-            <v>50.348585624999998</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="D26">
-            <v>50.348585624999998</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="D27">
-            <v>201.39434249999999</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="D28">
-            <v>302.09151374999999</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="D29">
-            <v>201.39434249999999</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="D30">
-            <v>2003.873707875</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="D31">
-            <v>5004.6494111250004</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="D32">
-            <v>2497.289847</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="D33">
-            <v>503.48585624999998</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="D34">
-            <v>302.09151374999999</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="D35">
-            <v>402.78868499999999</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="D36">
-            <v>151.045756875</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="D37">
-            <v>503.48585624999998</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="D38">
-            <v>3000.7757032499999</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="D39">
-            <v>2497.289847</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="D40">
-            <v>1198.2963378750001</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="D41">
-            <v>2497.289847</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="D42">
-            <v>3584.8192964999998</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -953,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51CCBCFD-2E22-41F3-84DE-C40DB9077DD2}">
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -997,13 +739,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1015,8 +757,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="1">
-        <f>[1]TK!D2</f>
-        <v>100.69717125</v>
+        <v>503.48585624999998</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1024,13 +765,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1042,7 +783,6 @@
         <v>0</v>
       </c>
       <c r="H3" s="1">
-        <f>[1]TK!D3</f>
         <v>201.39434249999999</v>
       </c>
     </row>
@@ -1051,13 +791,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -1069,8 +809,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="1">
-        <f>[1]TK!D4</f>
-        <v>201.39434249999999</v>
+        <v>12003.102813</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1078,13 +817,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -1096,8 +835,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="1">
-        <f>[1]TK!D5</f>
-        <v>201.39434249999999</v>
+        <v>45001.565831624997</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -1105,13 +843,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -1123,8 +861,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="1">
-        <f>[1]TK!D6</f>
-        <v>12003.102813</v>
+        <v>503.48585624999998</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -1132,13 +869,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -1150,8 +887,7 @@
         <v>0</v>
       </c>
       <c r="H7" s="1">
-        <f>[1]TK!D7</f>
-        <v>30007.757032499998</v>
+        <v>1500.3878516249999</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -1159,13 +895,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -1177,8 +913,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="1">
-        <f>[1]TK!D8</f>
-        <v>7995.3553972499994</v>
+        <v>5034.8585625000005</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1186,13 +921,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -1204,8 +939,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="1">
-        <f>[1]TK!D9</f>
-        <v>503.48585624999998</v>
+        <v>2003.873707875</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -1213,13 +947,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -1231,8 +965,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="1">
-        <f>[1]TK!D10</f>
-        <v>6998.453401875001</v>
+        <v>1500.3878516249999</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -1240,13 +973,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -1258,8 +991,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="1">
-        <f>[1]TK!D11</f>
-        <v>1500.3878516249999</v>
+        <v>503.48585624999998</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -1267,13 +999,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D12" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -1285,8 +1017,7 @@
         <v>0</v>
       </c>
       <c r="H12" s="1">
-        <f>[1]TK!D12</f>
-        <v>5034.8585625000005</v>
+        <v>805.57736999999997</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -1294,13 +1025,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -1312,8 +1043,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="1">
-        <f>[1]TK!D13</f>
-        <v>2003.873707875</v>
+        <v>3524.4009937500005</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -1321,26 +1051,25 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H14" s="1">
-        <f>[1]TK!D14</f>
-        <v>1500.3878516249999</v>
+        <v>302.09151374999999</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -1348,26 +1077,25 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H15" s="1">
-        <f>[1]TK!D15</f>
-        <v>503.48585624999998</v>
+        <v>1500.3878516249999</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -1375,26 +1103,25 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D16" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H16" s="1">
-        <f>[1]TK!D16</f>
-        <v>805.57736999999997</v>
+        <v>201.39434249999999</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -1402,26 +1129,25 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H17" s="1">
-        <f>[1]TK!D17</f>
-        <v>3524.4009937500005</v>
+        <v>402.78868499999999</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -1429,13 +1155,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="C18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D18" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -1444,11 +1170,10 @@
         <v>1</v>
       </c>
       <c r="G18" s="2">
-        <v>2.7000000000000001E-3</v>
+        <v>0.01</v>
       </c>
       <c r="H18" s="1">
-        <f>[1]TK!D18</f>
-        <v>302.09151374999999</v>
+        <v>50.348585624999998</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -1456,13 +1181,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="C19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D19" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -1471,11 +1196,10 @@
         <v>1</v>
       </c>
       <c r="G19" s="2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H19" s="1">
-        <f>[1]TK!D19</f>
-        <v>1500.3878516249999</v>
+        <v>100.69717125</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
@@ -1483,13 +1207,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D20" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -1498,11 +1222,10 @@
         <v>1</v>
       </c>
       <c r="G20" s="2">
-        <v>0.41808508590274895</v>
+        <v>0.01</v>
       </c>
       <c r="H20" s="1">
-        <f>[1]TK!D20</f>
-        <v>201.39434249999999</v>
+        <v>50.348585624999998</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -1510,13 +1233,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D21" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -1525,11 +1248,10 @@
         <v>1</v>
       </c>
       <c r="G21" s="2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H21" s="1">
-        <f>[1]TK!D21</f>
-        <v>100.69717125</v>
+        <v>50.348585624999998</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -1537,13 +1259,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C22" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D22" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -1552,11 +1274,10 @@
         <v>1</v>
       </c>
       <c r="G22" s="2">
-        <v>1.1474827820314282E-2</v>
+        <v>0.01</v>
       </c>
       <c r="H22" s="1">
-        <f>[1]TK!D22</f>
-        <v>402.78868499999999</v>
+        <v>302.09151374999999</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
@@ -1564,13 +1285,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="C23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D23" t="s">
-        <v>8</v>
+        <v>78</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -1579,11 +1300,10 @@
         <v>1</v>
       </c>
       <c r="G23" s="2">
-        <v>0.10204164174912744</v>
+        <v>0.01</v>
       </c>
       <c r="H23" s="1">
-        <f>[1]TK!D23</f>
-        <v>50.348585624999998</v>
+        <v>302.09151374999999</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
@@ -1591,13 +1311,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C24" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D24" t="s">
-        <v>8</v>
+        <v>79</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -1606,11 +1326,10 @@
         <v>1</v>
       </c>
       <c r="G24" s="2">
-        <v>0.2225185103524232</v>
+        <v>0.01</v>
       </c>
       <c r="H24" s="1">
-        <f>[1]TK!D24</f>
-        <v>100.69717125</v>
+        <v>201.39434249999999</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
@@ -1618,13 +1337,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D25" t="s">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -1633,11 +1352,10 @@
         <v>1</v>
       </c>
       <c r="G25" s="2">
-        <v>0.71908987139005265</v>
+        <v>0.01</v>
       </c>
       <c r="H25" s="1">
-        <f>[1]TK!D25</f>
-        <v>50.348585624999998</v>
+        <v>2003.873707875</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
@@ -1645,13 +1363,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D26" t="s">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -1660,11 +1378,10 @@
         <v>1</v>
       </c>
       <c r="G26" s="2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H26" s="1">
-        <f>[1]TK!D26</f>
-        <v>50.348585624999998</v>
+        <v>7501.9392581250004</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -1672,13 +1389,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="C27" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D27" t="s">
-        <v>8</v>
+        <v>81</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -1687,11 +1404,10 @@
         <v>1</v>
       </c>
       <c r="G27" s="2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H27" s="1">
-        <f>[1]TK!D27</f>
-        <v>201.39434249999999</v>
+        <v>805.57736999999997</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -1699,13 +1415,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="C28" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D28" t="s">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -1714,11 +1430,10 @@
         <v>1</v>
       </c>
       <c r="G28" s="2">
-        <v>6.9332659657442175E-2</v>
+        <v>0.01</v>
       </c>
       <c r="H28" s="1">
-        <f>[1]TK!D28</f>
-        <v>302.09151374999999</v>
+        <v>402.78868499999999</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
@@ -1726,13 +1441,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="C29" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D29" t="s">
-        <v>8</v>
+        <v>83</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1741,11 +1456,10 @@
         <v>1</v>
       </c>
       <c r="G29" s="2">
-        <v>0.20272920751195733</v>
+        <v>0.01</v>
       </c>
       <c r="H29" s="1">
-        <f>[1]TK!D29</f>
-        <v>201.39434249999999</v>
+        <v>151.045756875</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
@@ -1753,13 +1467,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="C30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D30" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -1768,11 +1482,10 @@
         <v>1</v>
       </c>
       <c r="G30" s="2">
-        <v>0.15619685398174643</v>
+        <v>0.01</v>
       </c>
       <c r="H30" s="1">
-        <f>[1]TK!D30</f>
-        <v>2003.873707875</v>
+        <v>503.48585624999998</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
@@ -1780,13 +1493,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D31" t="s">
-        <v>8</v>
+        <v>85</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -1795,11 +1508,10 @@
         <v>1</v>
       </c>
       <c r="G31" s="2">
-        <v>7.9160750938956248E-2</v>
+        <v>0.01</v>
       </c>
       <c r="H31" s="1">
-        <f>[1]TK!D31</f>
-        <v>5004.6494111250004</v>
+        <v>3000.7757032499999</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
@@ -1807,13 +1519,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="C32" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D32" t="s">
-        <v>8</v>
+        <v>86</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -1822,10 +1534,9 @@
         <v>1</v>
       </c>
       <c r="G32" s="2">
-        <v>3.3716767936662118E-2</v>
+        <v>0.01</v>
       </c>
       <c r="H32" s="1">
-        <f>[1]TK!D32</f>
         <v>2497.289847</v>
       </c>
     </row>
@@ -1834,13 +1545,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="C33" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D33" t="s">
-        <v>8</v>
+        <v>87</v>
       </c>
       <c r="E33">
         <v>0</v>
@@ -1849,11 +1560,10 @@
         <v>1</v>
       </c>
       <c r="G33" s="2">
-        <v>5.6907034608510099E-2</v>
+        <v>0.01</v>
       </c>
       <c r="H33" s="1">
-        <f>[1]TK!D33</f>
-        <v>503.48585624999998</v>
+        <v>1198.2963378750001</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
@@ -1861,13 +1571,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="C34" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D34" t="s">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="E34">
         <v>0</v>
@@ -1876,11 +1586,10 @@
         <v>1</v>
       </c>
       <c r="G34" s="2">
-        <v>0.12868594096542441</v>
+        <v>0.01</v>
       </c>
       <c r="H34" s="1">
-        <f>[1]TK!D34</f>
-        <v>302.09151374999999</v>
+        <v>2497.289847</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
@@ -1888,13 +1597,13 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="C35" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="E35">
         <v>0</v>
@@ -1903,199 +1612,9 @@
         <v>1</v>
       </c>
       <c r="G35" s="2">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="H35" s="1">
-        <f>[1]TK!D35</f>
-        <v>402.78868499999999</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36" t="s">
-        <v>83</v>
-      </c>
-      <c r="C36" t="s">
-        <v>43</v>
-      </c>
-      <c r="D36" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36">
-        <v>0</v>
-      </c>
-      <c r="F36">
-        <v>1</v>
-      </c>
-      <c r="G36" s="2">
-        <v>0.18185073335734003</v>
-      </c>
-      <c r="H36" s="1">
-        <f>[1]TK!D36</f>
-        <v>151.045756875</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37" t="s">
-        <v>84</v>
-      </c>
-      <c r="C37" t="s">
-        <v>44</v>
-      </c>
-      <c r="D37" t="s">
-        <v>8</v>
-      </c>
-      <c r="E37">
-        <v>0</v>
-      </c>
-      <c r="F37">
-        <v>1</v>
-      </c>
-      <c r="G37" s="2">
-        <v>4.424127182093418E-2</v>
-      </c>
-      <c r="H37" s="1">
-        <f>[1]TK!D37</f>
-        <v>503.48585624999998</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38" t="s">
-        <v>85</v>
-      </c>
-      <c r="C38" t="s">
-        <v>45</v>
-      </c>
-      <c r="D38" t="s">
-        <v>8</v>
-      </c>
-      <c r="E38">
-        <v>0</v>
-      </c>
-      <c r="F38">
-        <v>1</v>
-      </c>
-      <c r="G38" s="2">
-        <v>9.8798245163341791E-2</v>
-      </c>
-      <c r="H38" s="1">
-        <f>[1]TK!D38</f>
-        <v>3000.7757032499999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39" t="s">
-        <v>86</v>
-      </c>
-      <c r="C39" t="s">
-        <v>46</v>
-      </c>
-      <c r="D39" t="s">
-        <v>8</v>
-      </c>
-      <c r="E39">
-        <v>0</v>
-      </c>
-      <c r="F39">
-        <v>1</v>
-      </c>
-      <c r="G39" s="2">
-        <v>6.5439809491808498E-2</v>
-      </c>
-      <c r="H39" s="1">
-        <f>[1]TK!D39</f>
-        <v>2497.289847</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40" t="s">
-        <v>87</v>
-      </c>
-      <c r="C40" t="s">
-        <v>47</v>
-      </c>
-      <c r="D40" t="s">
-        <v>8</v>
-      </c>
-      <c r="E40">
-        <v>0</v>
-      </c>
-      <c r="F40">
-        <v>1</v>
-      </c>
-      <c r="G40" s="2">
-        <v>7.826757953253205E-2</v>
-      </c>
-      <c r="H40" s="1">
-        <f>[1]TK!D40</f>
-        <v>1198.2963378750001</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" t="s">
-        <v>88</v>
-      </c>
-      <c r="C41" t="s">
-        <v>48</v>
-      </c>
-      <c r="D41" t="s">
-        <v>8</v>
-      </c>
-      <c r="E41">
-        <v>0</v>
-      </c>
-      <c r="F41">
-        <v>1</v>
-      </c>
-      <c r="G41" s="2">
-        <v>2.3900000000000001E-2</v>
-      </c>
-      <c r="H41" s="1">
-        <f>[1]TK!D41</f>
-        <v>2497.289847</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42" t="s">
-        <v>89</v>
-      </c>
-      <c r="C42" t="s">
-        <v>90</v>
-      </c>
-      <c r="D42" t="s">
-        <v>8</v>
-      </c>
-      <c r="E42">
-        <v>0</v>
-      </c>
-      <c r="F42">
-        <v>1</v>
-      </c>
-      <c r="G42" s="2">
-        <v>0</v>
-      </c>
-      <c r="H42" s="1">
-        <f>[1]TK!D42</f>
         <v>3584.8192964999998</v>
       </c>
     </row>

</xml_diff>

<commit_message>
revised import multiplier and produce chart LRC and bar chart GRP
</commit_message>
<xml_diff>
--- a/DeskripsiSektor.xlsx
+++ b/DeskripsiSektor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/Documents/GitHub/Regional-Economy-GGP-PNG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0D032CE-CAB2-4934-82A0-FD6136D6581B}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="8_{D05DDFA1-92DF-4CA7-B250-8152B3E9D77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0F2C8DD-0EAA-4BF2-BC49-C97213B1A020}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{E1C60AC3-C6A1-4F74-BF98-34B67247E69B}"/>
   </bookViews>
   <sheets>
     <sheet name="DeskripsiSektor" sheetId="1" r:id="rId1"/>
@@ -315,18 +315,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00000_);_(* \(#,##0.00000\);_(* &quot;-&quot;??_);_(@_)"/>
-  </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -352,17 +341,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1066,7 +1052,7 @@
         <v>1</v>
       </c>
       <c r="G14">
-        <v>0.01</v>
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H14" s="1">
         <v>302.09151374999999</v>
@@ -1092,7 +1078,7 @@
         <v>1</v>
       </c>
       <c r="G15">
-        <v>0.01</v>
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H15" s="1">
         <v>1500.3878516249999</v>
@@ -1118,7 +1104,7 @@
         <v>1</v>
       </c>
       <c r="G16">
-        <v>0.01</v>
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H16" s="1">
         <v>201.39434249999999</v>
@@ -1144,7 +1130,7 @@
         <v>1</v>
       </c>
       <c r="G17">
-        <v>0.01</v>
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H17" s="1">
         <v>402.78868499999999</v>
@@ -1169,8 +1155,8 @@
       <c r="F18">
         <v>1</v>
       </c>
-      <c r="G18" s="2">
-        <v>0.01</v>
+      <c r="G18">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H18" s="1">
         <v>50.348585624999998</v>
@@ -1195,8 +1181,8 @@
       <c r="F19">
         <v>1</v>
       </c>
-      <c r="G19" s="2">
-        <v>0.01</v>
+      <c r="G19">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H19" s="1">
         <v>100.69717125</v>
@@ -1221,8 +1207,8 @@
       <c r="F20">
         <v>1</v>
       </c>
-      <c r="G20" s="2">
-        <v>0.01</v>
+      <c r="G20">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H20" s="1">
         <v>50.348585624999998</v>
@@ -1247,8 +1233,8 @@
       <c r="F21">
         <v>1</v>
       </c>
-      <c r="G21" s="2">
-        <v>0.01</v>
+      <c r="G21">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H21" s="1">
         <v>50.348585624999998</v>
@@ -1273,8 +1259,8 @@
       <c r="F22">
         <v>1</v>
       </c>
-      <c r="G22" s="2">
-        <v>0.01</v>
+      <c r="G22">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H22" s="1">
         <v>302.09151374999999</v>
@@ -1299,8 +1285,8 @@
       <c r="F23">
         <v>1</v>
       </c>
-      <c r="G23" s="2">
-        <v>0.01</v>
+      <c r="G23">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H23" s="1">
         <v>302.09151374999999</v>
@@ -1325,8 +1311,8 @@
       <c r="F24">
         <v>1</v>
       </c>
-      <c r="G24" s="2">
-        <v>0.01</v>
+      <c r="G24">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H24" s="1">
         <v>201.39434249999999</v>
@@ -1351,8 +1337,8 @@
       <c r="F25">
         <v>1</v>
       </c>
-      <c r="G25" s="2">
-        <v>0.01</v>
+      <c r="G25">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H25" s="1">
         <v>2003.873707875</v>
@@ -1377,8 +1363,8 @@
       <c r="F26">
         <v>1</v>
       </c>
-      <c r="G26" s="2">
-        <v>0.01</v>
+      <c r="G26">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H26" s="1">
         <v>7501.9392581250004</v>
@@ -1403,8 +1389,8 @@
       <c r="F27">
         <v>1</v>
       </c>
-      <c r="G27" s="2">
-        <v>0.01</v>
+      <c r="G27">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H27" s="1">
         <v>805.57736999999997</v>
@@ -1429,8 +1415,8 @@
       <c r="F28">
         <v>1</v>
       </c>
-      <c r="G28" s="2">
-        <v>0.01</v>
+      <c r="G28">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H28" s="1">
         <v>402.78868499999999</v>
@@ -1455,8 +1441,8 @@
       <c r="F29">
         <v>1</v>
       </c>
-      <c r="G29" s="2">
-        <v>0.01</v>
+      <c r="G29">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H29" s="1">
         <v>151.045756875</v>
@@ -1481,8 +1467,8 @@
       <c r="F30">
         <v>1</v>
       </c>
-      <c r="G30" s="2">
-        <v>0.01</v>
+      <c r="G30">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H30" s="1">
         <v>503.48585624999998</v>
@@ -1507,8 +1493,8 @@
       <c r="F31">
         <v>1</v>
       </c>
-      <c r="G31" s="2">
-        <v>0.01</v>
+      <c r="G31">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H31" s="1">
         <v>3000.7757032499999</v>
@@ -1533,8 +1519,8 @@
       <c r="F32">
         <v>1</v>
       </c>
-      <c r="G32" s="2">
-        <v>0.01</v>
+      <c r="G32">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H32" s="1">
         <v>2497.289847</v>
@@ -1559,8 +1545,8 @@
       <c r="F33">
         <v>1</v>
       </c>
-      <c r="G33" s="2">
-        <v>0.01</v>
+      <c r="G33">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H33" s="1">
         <v>1198.2963378750001</v>
@@ -1585,8 +1571,8 @@
       <c r="F34">
         <v>1</v>
       </c>
-      <c r="G34" s="2">
-        <v>0.01</v>
+      <c r="G34">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H34" s="1">
         <v>2497.289847</v>
@@ -1611,8 +1597,8 @@
       <c r="F35">
         <v>1</v>
       </c>
-      <c r="G35" s="2">
-        <v>0.01</v>
+      <c r="G35">
+        <v>1.550737964398342E-2</v>
       </c>
       <c r="H35" s="1">
         <v>3584.8192964999998</v>

</xml_diff>